<commit_message>
Data save update for 3 platforms
</commit_message>
<xml_diff>
--- a/PromVesClient/Templates/CardTemplate.xlsx
+++ b/PromVesClient/Templates/CardTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Клиент\PromVesClient\PromVesClient\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E892DDC-73A8-43E5-8867-763974A9883D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4783EAD6-BFEF-4292-B7B5-FFA7BB863751}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,10 +60,10 @@
     <t>Недогруз перегруз, т.</t>
   </si>
   <si>
-    <t>АО «Уральский завод металлоконструкций»</t>
-  </si>
-  <si>
     <t>Грузоподъёмность, т.</t>
+  </si>
+  <si>
+    <t>ПАО «Химпром»</t>
   </si>
 </sst>
 </file>
@@ -448,7 +448,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -476,7 +476,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>

</xml_diff>